<commit_message>
Started to mark GDV5002 resits
</commit_message>
<xml_diff>
--- a/T2/GDV4000_PRAC1_Rubric.xlsx
+++ b/T2/GDV4000_PRAC1_Rubric.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ian\TEACHING_25_26\2025_26\T2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2025_26\T2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C5D1AFC-CA40-4C65-98AF-AB4AFB401BF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A63B987-929D-45ED-BD75-2A31C780EC0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{10AB7DF0-9F58-4F22-B422-EFDDE15238C8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="46296" windowHeight="25416" xr2:uid="{10AB7DF0-9F58-4F22-B422-EFDDE15238C8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="81">
   <si>
     <t>100% - 90%</t>
   </si>
@@ -113,47 +113,7 @@
     <t>No meaningful implementation is given. What has been implemented does not reflect the original design.</t>
   </si>
   <si>
-    <t>Little to no testing has been attempted. In addition, no reflection or meaningful changes have been proposed to the original design.</t>
-  </si>
-  <si>
     <t>No use of version control has been made and there is no evidence of project management throughout the assignment.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">An outstanding implementation is given that uses an array of techniques discussed in lectures, as well as the students' own research. The implemented game accurately reflects the design will all features covered. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">An excellent implementation is given that uses an excellent range of techniques discussed in lectures. The implemented game accurately reflects the design will all features covered. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">A very good implementation is given that uses a good range of techniques discussed in lectures. The implemented game closely reflects the design, with most features covered. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">A good implementation is given that uses a number of techniques discussed in lectures, but the range of techniques used could be expanded. The implemented game reflects the design in many respects, in particular the high priority / core “must have” features, but closer attention to other aspects of the design is needed. </t>
-  </si>
-  <si>
-    <t>A basic implementation is given that uses few techniques discussed in the lectures, but a wider range of techniques are needed to fully realise your design. The implemented game reflects some elements of the design, in particular the high priority
-/ core “must have” features, but closer attention to other aspects of the design is needed.</t>
-  </si>
-  <si>
-    <t>A very basic implementation is given that uses only a few of the techniques discussed in the lectures. This needs to be significantly expanded. The implemented game does not resemble the design. In addition, little to no attention has been paid to the core / high priority “must have” features set out in the design.</t>
-  </si>
-  <si>
-    <t>A complete range of testing has been undertaken and an outstanding written reflection produced on the original design and what needs to be changed is evident. A highly detailed re-design has been completed based on the feedback obtained.</t>
-  </si>
-  <si>
-    <t>Thorough testing has been done and an excellent written reflection on the original design and what needs to be changed is evident. A detailed re-design has been completed based on the feedback obtained.</t>
-  </si>
-  <si>
-    <t>A very good range of testing has been done and a well written reflection on the original design and what needs to be changed is also given, but there is scope for these to be expanded upon. A proposed re-design is given but this could be more detailed – you need to elaborate on which core / non-core features have changed.</t>
-  </si>
-  <si>
-    <t>A good range of testing has been done and a good reflection on the original design and what needs to be changed is evident, but these need to be expanded further. A proposed re-design is given based on the testing feedback obtained, but this could be more detailed – in particular you need to elaborate on which core / non-core features have changed.</t>
-  </si>
-  <si>
-    <t>Basic testing has been done and an overview of what needs to be changed is evident. However, these need to be expanded further and more reflection is needed as well as further justification for the proposed changes.</t>
-  </si>
-  <si>
-    <t>Little to no testing has been done and no reflection or proposed changes to the design are evident.</t>
   </si>
   <si>
     <t>The appendices show little to no use of or understanding of version control systems. In addition, little to no project management is evident – you need to better plan and manage meetings and document activities more thoroughly</t>
@@ -174,6 +134,154 @@
   <si>
     <t>A very detailed set of appendices are given showing excellent use of and understanding of version control systems.
 Outstanding project management skills are also evident with clear, well documented activities and meetings given.</t>
+  </si>
+  <si>
+    <t>Part 1 - Implementation</t>
+  </si>
+  <si>
+    <t>Part 2 - Report (TDD)</t>
+  </si>
+  <si>
+    <t>Part 3 - Presentation</t>
+  </si>
+  <si>
+    <t>Part 4 - Reflective Report</t>
+  </si>
+  <si>
+    <t>An outstanding implementation is given that uses an array of techniques discussed in lectures, as well as the students' own research. The implemented game accurately reflects the design will all features covered. Scale has been considered and the level/ environment works and is fully playable.</t>
+  </si>
+  <si>
+    <t>An excellent implementation is given that uses an excellent range of techniques discussed in lectures. The implemented game accurately reflects the design will all features covered. Scale has been considered and the level/ environment works and is fully playable.</t>
+  </si>
+  <si>
+    <t>A very good implementation is given that uses a good range of techniques discussed in lectures. The implemented game closely reflects the design, with most features covered. Scale has been considered and the level/ environment works and the main gameloop is playable.</t>
+  </si>
+  <si>
+    <t>A good implementation is given that uses a number of techniques discussed in lectures, but the range of techniques used could be expanded. The implemented game reflects the design in many respects, in particular the high priority / core “must have” features, but closer attention to other aspects of the design is needed. Scale has been largely considered. and the level/ environment mostly works and is playable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A basic implementation is given that uses few techniques discussed in the lectures, but a wider range of techniques are needed to fully realise your design. The implemented game reflects some elements of the design, in particular the high priority
+/ core “must have” features, but closer attention to other aspects of the design is needed. Scale has been considered but is inconsistent. The level/ environment works in part and there is some degree of  playability. </t>
+  </si>
+  <si>
+    <t>A very basic implementation is given that uses only a few of the techniques discussed in the lectures. This needs to be significantly expanded. The implemented game does not resemble the design. In addition, little to no attention has been paid to the core / high priority “must have” features set out in the design. Scale has not been considered and the level/ environment works is not fully playable.</t>
+  </si>
+  <si>
+    <t>Outstanding thought has been given. GameObjects/Actors have been created with OOP principles, inheritance, and polymorphism in mind. Singeton patterns can be used in the prototype, but some concept of creating systems have been demonstrated.</t>
+  </si>
+  <si>
+    <t>An outstanding presentation that includes all group members. It shows clear evidence of having been well-prepared and rehearsed. It comes in on time, with a 10% margin either way. A complete range of testing has been undertaken and an outstanding written reflection produced on the original design and what needs to be changed is evident. A highly detailed re-design has been completed based on the feedback obtained.</t>
+  </si>
+  <si>
+    <t>An outstanding range of assets have been created (character, NPC, environment, UI...) with the appropriate texture/modelling formats in place. If pre-existing assets have been used, these have been credited/referenced, and the appropriate licence used. Pre-existed assets have been selected or modified to resemble descriptions/concept art in the GDD. A file structure has been implemented in the engine to accommodate all assets and relevant components.</t>
+  </si>
+  <si>
+    <t>A excellent range of assets have been created (character, NPC, environment, UI...) with the appropriate texture/modelling formats in place. If pre-existing assets have been used, these have been credited/referenced, and the appropriate licence used. Pre-existed assets have been selected or modified to resemble descriptions/concept art in the GDD. A file structure has been implemented in the engine to accommodate all assets and relevant components.</t>
+  </si>
+  <si>
+    <t>A good range of assets have been created (character, NPC, environment, UI...) with the appropriate texture/modelling formats in place. If pre-existing assets have been used, these have been credited/referenced, and the appropriate licence used. Pre-existed assets have been used but little modification made to resemble descriptions/concept art in the GDD. A loose file structure has been implemented in the engine to accommodate all assets and relevant components.</t>
+  </si>
+  <si>
+    <t>A very good of assets have been created (character, NPC, environment, UI...) with the appropriate texture/modelling formats in place, but leaning more toward placeholder and pre-existing assets. Pre-existing assets have been mostly credited/referenced, and the appropriate licence used. Pre-existed assets have been selected or  modified in some way to resemble descriptions/concept art in the GDD. A file structure has been implemented in the engine to accommodate all assets and relevant components.</t>
+  </si>
+  <si>
+    <t>A small range of assets have been created (character, NPC, environment, UI...) with the appropriate texture/modelling formats in place. Pre-existing assets have been used, but have not been credited/referenced, nor have the appropriate licences been used. Pre-existed assets have not been selected or modified to resemble descriptions/concept art in the GDD. A very loose and indistinct file structure has been implemented in the engine to accommodate all assets and relevant components.</t>
+  </si>
+  <si>
+    <t>Very few assets have been created and few, if any, pre-existing assets have been used, these have been credited/referenced, and the appropriate licence used. Pre-existed assets do not resemble descriptions/concept art in the GDD. No structure has been implemented in the engine to accommodate all assets and relevant components.</t>
+  </si>
+  <si>
+    <t>No assets have been created and few, if any, pre-existing assets have been used, these have been credited/referenced, and the appropriate licence used. Pre-existed assets do not resemble descriptions/concept art in the GDD. No structure has been implemented in the engine to accommodate all assets and relevant components.</t>
+  </si>
+  <si>
+    <t>Excellent thought has been given. GameObjects/Actors have been created with OOP principles, inheritance, and polymorphism in mind. Singeton patterns can be used in the prototype, at least one concept of creating a system has been demonstrated.</t>
+  </si>
+  <si>
+    <t>Very good level of thought has been given. GameObjects/Actors have largely been created with OOP principles, inheritance, and polymorphism in mind. Singeton patterns have been used throughout the prototype.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A good level of thought has been given. GameObjects/Actors have been created with some understanding of OOP principles, inheritance, and polymorphism in mind. Singeton patterns have been used. Some evidence of using tutorials but not fully understanding the logic driving the code, where it repeats or is unoptimised. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">A basic level of thought has been given. GameObjects/Actors have been created with little understanding of OOP principles, inheritance, and polymorphism in mind. Mostly Singeton patterns have been used. Some evidence of using tutorials and largely not  understanding the logic driving the code, where it repeats or is unoptimised. </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> GameObjects/Actors have been created with little to no understanding of OOP principles, inheritance, and polymorphism in mind. Singeton patterns have been used. Some evidence of using tutorials but not fully understanding the logic driving the code, where it repeats or is unoptimised. </t>
+  </si>
+  <si>
+    <t>An excellent range of different Actor/GameObjects using a variety of collisions and triggers to fire different actions. These actions can be fully realised, or they can be a debug message to the log. Inheritance and the idea of using systems over Singleton patterns is evident.</t>
+  </si>
+  <si>
+    <t>Outstanding range of different Actor/GameObjects using a variety of collisions and triggers to fire different actions. These actions are fully realised, or they can be a debug message to the log. Inheritance and the idea of using systems over Singleton patterns is evident.</t>
+  </si>
+  <si>
+    <t>A good range of different Actor/GameObjects using a one or two different types of collisions and triggers to fire different actions. These are largely a debug message to the log. Some notion of inheretance, but largely Singleton patterns.</t>
+  </si>
+  <si>
+    <t>A very good range of different Actor/GameObjects using a few different types of collisions and triggers to fire different actions. A few of these actions are fully realised, but they are largely a debug message to the log. Some notion of inheretance, but largely Singleton patterns.</t>
+  </si>
+  <si>
+    <t>A basic range of different Actor/GameObjects using a one types of collision or trigger to fire an action, resulting in a debug message to the log.</t>
+  </si>
+  <si>
+    <t>No behaviours demonstrated. No evidence of triggers or collision events used.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project management tools or concepts used (screenshots of Trello, Jisc, Gannt charts - use of some colour coding to denote priority or type of mechanic, gameplay event...). Full details of allocation of tasks, including a rationale for how these tasks were selected and prioritised from the GDD, with a clear idea of what was needing to be produced.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project management tools or concepts used (screenshots of Trello, Jisc, Gannt charts). Details of allocation of tasks, including a rationale for how these tasks were selected and prioritised from the GDD is largely present, with a very good understanding of what was needing to be produced.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project management tools or concepts used (screenshots of Trello, Jisc, Gannt charts). Full details of allocation of tasks, including a rationale for how these tasks were selected and prioritised from the GDD, with an excellent idea of what was needing to be produced.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Some evidence of a  management tool or concept used (screenshots of Trello, Jisc, Gannt charts). Some details of allocation of tasks, including a rationale for how these tasks were selected and prioritised from the GDD is largely present, with a good understanding of what was needing to be produced.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Little evidence of a  management tool or concept used (screenshots of Trello, Jisc, Gannt charts). Some details of allocation of tasks, including a rationale for how these tasks were selected and prioritised from the GDD is largely present, with a basic understanding of what was needing to be produced.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No management tools used No allocation of tasks, Little to no understanding of what was needing to be produced is evident.  </t>
+  </si>
+  <si>
+    <t>Excellent overview that gives each group member the opportunity to perform a short code demo of a system or feature that they were responsible for, and how it was implemented in the game engine. Code/scripts/and visual scripting should be well explained and demonstrate that the students understands the core logic behind it, with recommendations for improvement if appropriate.</t>
+  </si>
+  <si>
+    <t>Outstanding overview that gives each group member the opportunity to perform a short code demo of a system or feature that they were responsible for, and how it was implemented in the game engine. Code/scripts/and visual scripting should be very well explained and demonstrate that the students understands the core logic behind it, with recommendations for improvement if appropriate.</t>
+  </si>
+  <si>
+    <t>A very good overview that gives each group member the opportunity to perform a short code demo of a system or feature that they were responsible for, and how it was implemented in the game engine. Code/scripts/and visual scripting should be explained and demonstrate that the students understands most of the core logic behind it, with some recommendations for improvement if appropriate.</t>
+  </si>
+  <si>
+    <t>A  good overview that gives most  group members the opportunity to perform a short code demo of a system or feature that they were responsible for, and how it was implemented in the game engine. Code/scripts/and visual scripting should be explained to a satisfactory degree, and demonstrate that the students understands some of the core logic behind it, with a recommendation for improvement if appropriate.</t>
+  </si>
+  <si>
+    <t>A  basic overview that gives most or some of the group members the opportunity to perform a short code demo of a system or feature that they were responsible for, and how it was implemented in the game engine. Code/scripts/and visual scripting should be explained to a satisfactory degree, and demonstrate that the students understands some of the core logic behind it, with a recommendation for improvement if appropriate.</t>
+  </si>
+  <si>
+    <t>A very  basic overview that gives most or some of the group members the opportunity to perform a short code demo of a system or feature that they were responsible for, and how it was implemented in the game engine. Code/scripts/and visual scripting are not fully explained, or demonstrate little understanding of the logic driving it. No recommendations for improvements suggested.</t>
+  </si>
+  <si>
+    <t>No presentation given or code demo.</t>
+  </si>
+  <si>
+    <t>An excellent presentation that includes all group members. It shows clear evidence of having been well-prepared and rehearsed. It comes in on time, with a 10% margin either way. Thorough testing has been done and an excellent written reflection on the original design and what needs to be changed is evident. A detailed re-design has been completed based on the feedback obtained.</t>
+  </si>
+  <si>
+    <t>A basic presentation that includes all some members. It shows little evidence of having been well-prepared and rehearsed. It comes in over or under time (5-7 minutes). Basic testing has been done and an overview of what needs to be changed is evident. However, these need to be expanded further and more reflection is needed as well as further justification for the proposed changes.</t>
+  </si>
+  <si>
+    <t>A good presentation that includes most group members. It shows some evidence of having been prepared and some  rehearsal. It comes in over or under time (3-4 minutes). A good range of testing has been done and a good reflection on the original design and what needs to be changed is evident, but these need to be expanded further. A proposed re-design is given based on the testing feedback obtained, but this could be more detailed – in particular you need to elaborate on which core / non-core features have changed.</t>
+  </si>
+  <si>
+    <t>A very good presentation that includes all group members. It shows good evidence of having been well-prepared and rehearsed. It comes in just over or under time (2-3 minutes). A very good range of testing has been done and a well written reflection on the original design and what needs to be changed is also given, but there is scope for these to be expanded upon. A proposed re-design is given but this could be more detailed – you need to elaborate on which core / non-core features have changed.</t>
+  </si>
+  <si>
+    <t>A very basic presentation that includes all few members. It shows little to no evidence of having been well-prepared and rehearsed. It comes in well over or under time (7+ minutes). Little to no testing has been done and no reflection or proposed changes to the design are evident.</t>
+  </si>
+  <si>
+    <t>No presentation given. Little to no testing has been attempted. In addition, no reflection or meaningful changes have been proposed to the original design.</t>
   </si>
 </sst>
 </file>
@@ -195,12 +303,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -215,7 +329,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -234,6 +348,16 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -569,21 +693,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36D68E70-80C2-4C70-80FD-0280BCC74744}">
-  <dimension ref="A1:M13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="83.7109375" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" customWidth="1"/>
-    <col min="5" max="5" width="17.5703125" customWidth="1"/>
-    <col min="6" max="6" width="19.140625" customWidth="1"/>
-    <col min="7" max="7" width="20.42578125" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" customWidth="1"/>
+    <col min="1" max="1" width="83.6640625" customWidth="1"/>
+    <col min="2" max="2" width="25.88671875" customWidth="1"/>
+    <col min="3" max="3" width="23.6640625" customWidth="1"/>
+    <col min="4" max="4" width="23.21875" customWidth="1"/>
+    <col min="5" max="5" width="22.6640625" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="24.5546875" customWidth="1"/>
+    <col min="8" max="9" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
@@ -613,216 +736,320 @@
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+    </row>
+    <row r="3" spans="1:13" ht="297.60000000000002" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-    </row>
-    <row r="3" spans="1:13" ht="345" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="B3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="298.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B4" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="216" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="189.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+    </row>
+    <row r="8" spans="1:13" ht="194.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-    </row>
-    <row r="8" spans="1:13" ht="225" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C8" s="4" t="s">
+      <c r="G9" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+    </row>
+    <row r="11" spans="1:13" ht="316.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-    </row>
-    <row r="10" spans="1:13" ht="330" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="C11" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="259.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-    </row>
-    <row r="13" spans="1:13" ht="300" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+    </row>
+    <row r="14" spans="1:13" ht="244.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B14" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F14" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G14" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H14" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I14" s="5" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>